<commit_message>
substitui tábuas de mortalidade no Brasil para 2023
</commit_message>
<xml_diff>
--- a/data/raw/female_life_table_central_west_brazil_2025.xlsx
+++ b/data/raw/female_life_table_central_west_brazil_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6671f81417a0f489/Documentos/Projeto IC - Vanessa/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6671f81417a0f489/Documentos/projeto_longevidade/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_F25DC773A252ABDACC104828F1DA7B125ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C16E97F6-B748-44F4-8303-6DF6BE8B50A6}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_F25DC773A252ABDACC104828F1DA7B125ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{353F74B0-1093-4629-8BD4-07953C126A9C}"/>
   <bookViews>
-    <workbookView xWindow="6108" yWindow="3708" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -516,31 +516,31 @@
         <v>0</v>
       </c>
       <c r="B2" s="4">
-        <v>1.13120143385092E-2</v>
+        <v>1.1726854771632499E-2</v>
       </c>
       <c r="C2" s="4">
-        <v>8.3587855608104403E-2</v>
+        <v>8.4807003876639003E-2</v>
       </c>
       <c r="D2" s="4">
-        <v>1.11959518693688E-2</v>
+        <v>1.1602334625547E-2</v>
       </c>
       <c r="E2" s="5">
         <v>100000</v>
       </c>
       <c r="F2" s="5">
-        <v>1119.5951869368901</v>
+        <v>1160.2334625547101</v>
       </c>
       <c r="G2" s="5">
-        <v>98973.989373888297</v>
+        <v>98938.162461201995</v>
       </c>
       <c r="H2" s="6">
-        <v>0.98783594977837597</v>
+        <v>0.98740222290591795</v>
       </c>
       <c r="I2" s="5">
-        <v>8026721.1822285904</v>
+        <v>7988430.1035428699</v>
       </c>
       <c r="J2" s="7">
-        <v>80.267211822285901</v>
+        <v>79.884301035428706</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -548,31 +548,31 @@
         <v>1</v>
       </c>
       <c r="B3" s="4">
-        <v>5.8638319920598396E-4</v>
+        <v>6.0526361625415901E-4</v>
       </c>
       <c r="C3" s="4">
-        <v>1.5057755772792201</v>
+        <v>1.50511421024931</v>
       </c>
       <c r="D3" s="4">
-        <v>2.3421072979166002E-3</v>
+        <v>2.4174040311941299E-3</v>
       </c>
       <c r="E3" s="5">
-        <v>98880.404813063098</v>
+        <v>98839.766537445306</v>
       </c>
       <c r="F3" s="5">
-        <v>231.58851773361701</v>
+        <v>238.93565006990701</v>
       </c>
       <c r="G3" s="5">
-        <v>394943.98551530001</v>
+        <v>394762.948991757</v>
       </c>
       <c r="H3" s="6">
-        <v>0.99798112284349905</v>
+        <v>0.99790940864315003</v>
       </c>
       <c r="I3" s="5">
-        <v>7927747.1928546997</v>
+        <v>7889491.9410816599</v>
       </c>
       <c r="J3" s="7">
-        <v>80.175108585390504</v>
+        <v>79.821029707640406</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -580,31 +580,31 @@
         <v>5</v>
       </c>
       <c r="B4" s="4">
-        <v>2.4273087419677999E-4</v>
+        <v>2.52016129032258E-4</v>
       </c>
       <c r="C4" s="4">
-        <v>2.2981685044510098</v>
+        <v>2.3005087879744299</v>
       </c>
       <c r="D4" s="4">
-        <v>1.2128589563448701E-3</v>
+        <v>1.25922397579218E-3</v>
       </c>
       <c r="E4" s="5">
-        <v>98648.816295329496</v>
+        <v>98600.830887375399</v>
       </c>
       <c r="F4" s="5">
-        <v>119.64710037662</v>
+        <v>124.160530286419</v>
       </c>
       <c r="G4" s="5">
-        <v>492920.81517249899</v>
+        <v>492668.98417648801</v>
       </c>
       <c r="H4" s="6">
-        <v>0.99888194332797597</v>
+        <v>0.99883587958220299</v>
       </c>
       <c r="I4" s="5">
-        <v>7532803.2073394004</v>
+        <v>7494728.9920899104</v>
       </c>
       <c r="J4" s="7">
-        <v>76.359793155430296</v>
+        <v>76.0108096923706</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -612,31 +612,31 @@
         <v>10</v>
       </c>
       <c r="B5" s="4">
-        <v>2.34142012669489E-4</v>
+        <v>2.4429544155101602E-4</v>
       </c>
       <c r="C5" s="4">
-        <v>2.6046704538968899</v>
+        <v>2.6052105309018398</v>
       </c>
       <c r="D5" s="4">
-        <v>1.1700538418317099E-3</v>
+        <v>1.22076301725846E-3</v>
       </c>
       <c r="E5" s="5">
-        <v>98529.169194952905</v>
+        <v>98476.670357088995</v>
       </c>
       <c r="F5" s="5">
-        <v>115.284432949033</v>
+        <v>120.216677234683</v>
       </c>
       <c r="G5" s="5">
-        <v>492369.70176631602</v>
+        <v>492095.458152793</v>
       </c>
       <c r="H5" s="6">
-        <v>0.99845745187026302</v>
+        <v>0.99839259312641604</v>
       </c>
       <c r="I5" s="5">
-        <v>7039882.3921669004</v>
+        <v>7002060.00791342</v>
       </c>
       <c r="J5" s="7">
-        <v>71.449728539145298</v>
+        <v>71.103744496265506</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -644,31 +644,31 @@
         <v>15</v>
       </c>
       <c r="B6" s="4">
-        <v>4.0210486581308699E-4</v>
+        <v>4.1861288566573499E-4</v>
       </c>
       <c r="C6" s="4">
-        <v>2.6769087830318399</v>
+        <v>2.67678181964239</v>
       </c>
       <c r="D6" s="4">
-        <v>2.0086479981789099E-3</v>
+        <v>2.0910308400577502E-3</v>
       </c>
       <c r="E6" s="5">
-        <v>98413.8847620038</v>
+        <v>98356.453679854298</v>
       </c>
       <c r="F6" s="5">
-        <v>197.67885262019999</v>
+        <v>205.66637796328001</v>
       </c>
       <c r="G6" s="5">
-        <v>491610.19780371699</v>
+        <v>491304.460530899</v>
       </c>
       <c r="H6" s="6">
-        <v>0.99761984919188595</v>
+        <v>0.99752038489268402</v>
       </c>
       <c r="I6" s="5">
-        <v>6547512.6904005902</v>
+        <v>6509964.5497606304</v>
       </c>
       <c r="J6" s="7">
-        <v>66.530375324930603</v>
+        <v>66.187467178821393</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -676,31 +676,31 @@
         <v>20</v>
       </c>
       <c r="B7" s="4">
-        <v>5.4955619275963105E-4</v>
+        <v>5.7313264496118305E-4</v>
       </c>
       <c r="C7" s="4">
-        <v>2.6219660335741501</v>
+        <v>2.6227874485834102</v>
       </c>
       <c r="D7" s="4">
-        <v>2.7441946765070098E-3</v>
+        <v>2.8617641909543601E-3</v>
       </c>
       <c r="E7" s="5">
-        <v>98216.2059093836</v>
+        <v>98150.787301891003</v>
       </c>
       <c r="F7" s="5">
-        <v>269.524389403246</v>
+        <v>280.88440841455298</v>
       </c>
       <c r="G7" s="5">
-        <v>490440.09139413701</v>
+        <v>490086.21456827503</v>
       </c>
       <c r="H7" s="6">
-        <v>0.99681858635898002</v>
+        <v>0.99667766037236605</v>
       </c>
       <c r="I7" s="5">
-        <v>6055902.4925968703</v>
+        <v>6018660.08922973</v>
       </c>
       <c r="J7" s="7">
-        <v>61.658892608661503</v>
+        <v>61.320548257219798</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -708,31 +708,31 @@
         <v>25</v>
       </c>
       <c r="B8" s="4">
-        <v>7.2606928046962298E-4</v>
+        <v>7.5904242515531604E-4</v>
       </c>
       <c r="C8" s="4">
-        <v>2.5952007237891102</v>
+        <v>2.59539336840239</v>
       </c>
       <c r="D8" s="4">
-        <v>3.6240186813398701E-3</v>
+        <v>3.7882977306335501E-3</v>
       </c>
       <c r="E8" s="5">
-        <v>97946.681519980397</v>
+        <v>97869.902893476494</v>
       </c>
       <c r="F8" s="5">
-        <v>354.96060360365698</v>
+        <v>370.76033102866501</v>
       </c>
       <c r="G8" s="5">
-        <v>488879.79859727301</v>
+        <v>488457.981716657</v>
       </c>
       <c r="H8" s="6">
-        <v>0.99601798033856404</v>
+        <v>0.99583914052318101</v>
       </c>
       <c r="I8" s="5">
-        <v>5565462.4012027299</v>
+        <v>5528573.8746614503</v>
       </c>
       <c r="J8" s="7">
-        <v>56.821347235408098</v>
+        <v>56.489009503553497</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -740,31 +740,31 @@
         <v>30</v>
       </c>
       <c r="B9" s="4">
-        <v>8.7422274243181201E-4</v>
+        <v>9.1287209217476403E-4</v>
       </c>
       <c r="C9" s="4">
-        <v>2.5908763164272601</v>
+        <v>2.59002415710607</v>
       </c>
       <c r="D9" s="4">
-        <v>4.3619270109497496E-3</v>
+        <v>4.55434091227959E-3</v>
       </c>
       <c r="E9" s="5">
-        <v>97591.720916376697</v>
+        <v>97499.1425624478</v>
       </c>
       <c r="F9" s="5">
-        <v>425.68796351020899</v>
+        <v>444.04433388433199</v>
       </c>
       <c r="G9" s="5">
-        <v>486933.06962717901</v>
+        <v>486425.57669440401</v>
       </c>
       <c r="H9" s="6">
-        <v>0.99506724659790402</v>
+        <v>0.99485729288967295</v>
       </c>
       <c r="I9" s="5">
-        <v>5076582.6026054602</v>
+        <v>5040115.8929447997</v>
       </c>
       <c r="J9" s="7">
-        <v>52.018578573436798</v>
+        <v>51.693950946457001</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -772,31 +772,31 @@
         <v>35</v>
       </c>
       <c r="B10" s="4">
-        <v>1.13296569686315E-3</v>
+        <v>1.18003850346763E-3</v>
       </c>
       <c r="C10" s="4">
-        <v>2.63366622715668</v>
+        <v>2.6333751716642202</v>
       </c>
       <c r="D10" s="4">
-        <v>5.6496818286206896E-3</v>
+        <v>5.8837608887587402E-3</v>
       </c>
       <c r="E10" s="5">
-        <v>97166.032952866502</v>
+        <v>97055.098228563496</v>
       </c>
       <c r="F10" s="5">
-        <v>548.95717073297396</v>
+        <v>571.048991011863</v>
       </c>
       <c r="G10" s="5">
-        <v>484531.14887138299</v>
+        <v>483924.03242249199</v>
       </c>
       <c r="H10" s="6">
-        <v>0.99311375626207998</v>
+        <v>0.99282326264305598</v>
       </c>
       <c r="I10" s="5">
-        <v>4589649.5329782804</v>
+        <v>4553690.3162503904</v>
       </c>
       <c r="J10" s="7">
-        <v>47.235123154658702</v>
+        <v>46.918610143760901</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -804,31 +804,31 @@
         <v>40</v>
       </c>
       <c r="B11" s="4">
-        <v>1.6795190380719199E-3</v>
+        <v>1.75214666976097E-3</v>
       </c>
       <c r="C11" s="4">
-        <v>2.6603722239769501</v>
+        <v>2.6607732690805799</v>
       </c>
       <c r="D11" s="4">
-        <v>8.3647264212109006E-3</v>
+        <v>8.7249725800423294E-3</v>
       </c>
       <c r="E11" s="5">
-        <v>96617.075782133601</v>
+        <v>96484.049237551604</v>
       </c>
       <c r="F11" s="5">
-        <v>808.17540653493802</v>
+        <v>841.82068400908599</v>
       </c>
       <c r="G11" s="5">
-        <v>481194.54928163998</v>
+        <v>480451.03674108302</v>
       </c>
       <c r="H11" s="6">
-        <v>0.98973801166122399</v>
+        <v>0.98928979249265303</v>
       </c>
       <c r="I11" s="5">
-        <v>4105118.3841069001</v>
+        <v>4069766.2838279</v>
       </c>
       <c r="J11" s="7">
-        <v>42.488538913801598</v>
+        <v>42.180716045693799</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -836,31 +836,31 @@
         <v>45</v>
       </c>
       <c r="B12" s="4">
-        <v>2.4878541970281302E-3</v>
+        <v>2.5980995261904202E-3</v>
       </c>
       <c r="C12" s="4">
-        <v>2.6470022406004001</v>
+        <v>2.64688743872841</v>
       </c>
       <c r="D12" s="4">
-        <v>1.23668763378983E-2</v>
+        <v>1.2911561243760101E-2</v>
       </c>
       <c r="E12" s="5">
-        <v>95808.900375598605</v>
+        <v>95642.228553542504</v>
       </c>
       <c r="F12" s="5">
-        <v>1184.8568230150599</v>
+        <v>1234.8904914587799</v>
       </c>
       <c r="G12" s="5">
-        <v>476256.53642822901</v>
+        <v>475305.30644046603</v>
       </c>
       <c r="H12" s="6">
-        <v>0.985322832594134</v>
+        <v>0.98467965476044195</v>
       </c>
       <c r="I12" s="5">
-        <v>3623923.8348252601</v>
+        <v>3589315.2470868202</v>
       </c>
       <c r="J12" s="7">
-        <v>37.824500861803301</v>
+        <v>37.528561403997799</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -868,31 +868,31 @@
         <v>50</v>
       </c>
       <c r="B13" s="4">
-        <v>3.4868430701339402E-3</v>
+        <v>3.6396313745248399E-3</v>
       </c>
       <c r="C13" s="4">
-        <v>2.6447618719389099</v>
+        <v>2.6440367633720299</v>
       </c>
       <c r="D13" s="4">
-        <v>1.7292205778120101E-2</v>
+        <v>1.8043437325766399E-2</v>
       </c>
       <c r="E13" s="5">
-        <v>94624.043552583593</v>
+        <v>94407.338062083698</v>
       </c>
       <c r="F13" s="5">
-        <v>1636.2584326690701</v>
+        <v>1703.4328874156499</v>
       </c>
       <c r="G13" s="5">
-        <v>469266.43951493403</v>
+        <v>468023.46505160403</v>
       </c>
       <c r="H13" s="6">
-        <v>0.97895726115035997</v>
+        <v>0.97806301700494802</v>
       </c>
       <c r="I13" s="5">
-        <v>3147667.2983970302</v>
+        <v>3114009.9406463499</v>
       </c>
       <c r="J13" s="7">
-        <v>33.264984038098497</v>
+        <v>32.984829405935898</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -900,31 +900,31 @@
         <v>55</v>
       </c>
       <c r="B14" s="4">
-        <v>5.1610806542639999E-3</v>
+        <v>5.37927175893004E-3</v>
       </c>
       <c r="C14" s="4">
-        <v>2.6603815611877399</v>
+        <v>2.6595629182571798</v>
       </c>
       <c r="D14" s="4">
-        <v>2.5497521730025199E-2</v>
+        <v>2.6561947931583198E-2</v>
       </c>
       <c r="E14" s="5">
-        <v>92987.785119914493</v>
+        <v>92703.905174668107</v>
       </c>
       <c r="F14" s="5">
-        <v>2370.9580717219401</v>
+        <v>2462.3963023039501</v>
       </c>
       <c r="G14" s="5">
-        <v>459391.78837732098</v>
+        <v>457756.44225748198</v>
       </c>
       <c r="H14" s="6">
-        <v>0.96837344433030903</v>
+        <v>0.96705701500118002</v>
       </c>
       <c r="I14" s="5">
-        <v>2678400.8588820901</v>
+        <v>2645986.4755947501</v>
       </c>
       <c r="J14" s="7">
-        <v>28.803792405939099</v>
+        <v>28.542341022304399</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -932,31 +932,31 @@
         <v>60</v>
       </c>
       <c r="B15" s="4">
-        <v>7.9283033757475106E-3</v>
+        <v>8.2612601052226408E-3</v>
       </c>
       <c r="C15" s="4">
-        <v>2.6690360635783601</v>
+        <v>2.66726526729264</v>
       </c>
       <c r="D15" s="4">
-        <v>3.8922211475910101E-2</v>
+        <v>4.05253237051484E-2</v>
       </c>
       <c r="E15" s="5">
-        <v>90616.827048192601</v>
+        <v>90241.508872364095</v>
       </c>
       <c r="F15" s="5">
-        <v>3527.00730564572</v>
+        <v>3657.0663586935798</v>
       </c>
       <c r="G15" s="5">
-        <v>444862.80840800703</v>
+        <v>442676.57864707999</v>
       </c>
       <c r="H15" s="6">
-        <v>0.95075590064742899</v>
+        <v>0.94886047066289103</v>
       </c>
       <c r="I15" s="5">
-        <v>2219009.0705047701</v>
+        <v>2188230.0333372601</v>
       </c>
       <c r="J15" s="7">
-        <v>24.487825747028701</v>
+        <v>24.248597576446301</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -964,31 +964,31 @@
         <v>65</v>
       </c>
       <c r="B16" s="4">
-        <v>1.25761495286983E-2</v>
+        <v>1.3040226008321699E-2</v>
       </c>
       <c r="C16" s="4">
-        <v>2.6512898009258099</v>
+        <v>2.6478039122728498</v>
       </c>
       <c r="D16" s="4">
-        <v>6.1076681087724301E-2</v>
+        <v>6.3260723212755304E-2</v>
       </c>
       <c r="E16" s="5">
-        <v>87089.819742546795</v>
+        <v>86584.442513670496</v>
       </c>
       <c r="F16" s="5">
-        <v>5319.1571464029303</v>
+        <v>5477.39445238802</v>
       </c>
       <c r="G16" s="5">
-        <v>422955.94007249898</v>
+        <v>420038.30676650698</v>
       </c>
       <c r="H16" s="6">
-        <v>0.92647403389605598</v>
+        <v>0.92415717730397695</v>
       </c>
       <c r="I16" s="5">
-        <v>1774146.2620967701</v>
+        <v>1745553.45469018</v>
       </c>
       <c r="J16" s="7">
-        <v>20.371454061352502</v>
+        <v>20.160128124802402</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -996,31 +996,31 @@
         <v>70</v>
       </c>
       <c r="B17" s="4">
-        <v>1.8585683915362E-2</v>
+        <v>1.9133451105958502E-2</v>
       </c>
       <c r="C17" s="4">
-        <v>2.66638069592593</v>
+        <v>2.6634926744879901</v>
       </c>
       <c r="D17" s="4">
-        <v>8.9065479545770807E-2</v>
+        <v>9.1573424501094902E-2</v>
       </c>
       <c r="E17" s="5">
-        <v>81770.662596143899</v>
+        <v>81107.048061282505</v>
       </c>
       <c r="F17" s="5">
-        <v>7282.94327690099</v>
+        <v>7427.2501421465304</v>
       </c>
       <c r="G17" s="5">
-        <v>391857.69595926697</v>
+        <v>388181.41594087699</v>
       </c>
       <c r="H17" s="6">
-        <v>0.88141096676295605</v>
+        <v>0.87822159140341705</v>
       </c>
       <c r="I17" s="5">
-        <v>1351190.32202427</v>
+        <v>1325515.14792368</v>
       </c>
       <c r="J17" s="7">
-        <v>16.524145446853499</v>
+        <v>16.342786226446702</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -1028,31 +1028,31 @@
         <v>75</v>
       </c>
       <c r="B18" s="4">
-        <v>3.3659196089516098E-2</v>
+        <v>3.4609846997471799E-2</v>
       </c>
       <c r="C18" s="4">
-        <v>2.6731329686914802</v>
+        <v>2.6701321264379301</v>
       </c>
       <c r="D18" s="4">
-        <v>0.156072322241153</v>
+        <v>0.160136415625863</v>
       </c>
       <c r="E18" s="5">
-        <v>74487.719319242897</v>
+        <v>73679.797919136006</v>
       </c>
       <c r="F18" s="5">
-        <v>11625.471332601401</v>
+        <v>11798.8187428084</v>
       </c>
       <c r="G18" s="5">
-        <v>345387.67062896199</v>
+        <v>340909.30086082901</v>
       </c>
       <c r="H18" s="6">
-        <v>0.79672387225017305</v>
+        <v>0.79202047266150599</v>
       </c>
       <c r="I18" s="5">
-        <v>959332.62606499996</v>
+        <v>937333.73198279901</v>
       </c>
       <c r="J18" s="7">
-        <v>12.879071004355101</v>
+        <v>12.721719636249899</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
@@ -1060,31 +1060,31 @@
         <v>80</v>
       </c>
       <c r="B19" s="4">
-        <v>5.9741194824998602E-2</v>
+        <v>6.1201447847599601E-2</v>
       </c>
       <c r="C19" s="4">
-        <v>2.6195966335617298</v>
+        <v>2.6158450964345401</v>
       </c>
       <c r="D19" s="4">
-        <v>0.26151623625373099</v>
+        <v>0.26704212603009297</v>
       </c>
       <c r="E19" s="5">
-        <v>62862.247986641501</v>
+        <v>61880.979176327601</v>
       </c>
       <c r="F19" s="5">
-        <v>16439.498495915199</v>
+        <v>16524.828240070499</v>
       </c>
       <c r="G19" s="5">
-        <v>275178.60237097403</v>
+        <v>270007.14560249698</v>
       </c>
       <c r="H19" s="6">
-        <v>0.66291676900500096</v>
+        <v>0.65611442438089196</v>
       </c>
       <c r="I19" s="5">
-        <v>613944.95543603797</v>
+        <v>596424.43112196994</v>
       </c>
       <c r="J19" s="7">
-        <v>9.7665128928654301</v>
+        <v>9.6382513505883693</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -1092,31 +1092,31 @@
         <v>85</v>
       </c>
       <c r="B20" s="4">
-        <v>0.10860984906188099</v>
+        <v>0.11129776511365801</v>
       </c>
       <c r="C20" s="4">
-        <v>2.4918447447314098</v>
+        <v>2.4831302794200298</v>
       </c>
       <c r="D20" s="4">
-        <v>0.42678782003231702</v>
+        <v>0.43471546965340702</v>
       </c>
       <c r="E20" s="5">
-        <v>46422.749490726303</v>
+        <v>45356.150936257203</v>
       </c>
       <c r="F20" s="5">
-        <v>19812.664055053399</v>
+        <v>19717.0204559259</v>
       </c>
       <c r="G20" s="5">
-        <v>182420.50998307799</v>
+        <v>177155.58291570999</v>
       </c>
       <c r="H20" s="6">
-        <v>0.46151526462829601</v>
+        <v>0.45727266669172301</v>
       </c>
       <c r="I20" s="5">
-        <v>338766.353065064</v>
+        <v>326417.28551947302</v>
       </c>
       <c r="J20" s="7">
-        <v>7.29742113040371</v>
+        <v>7.1967589573069199</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
@@ -1124,31 +1124,31 @@
         <v>90</v>
       </c>
       <c r="B21" s="4">
-        <v>0.170200146745947</v>
+        <v>0.171773000261119</v>
       </c>
       <c r="C21" s="4">
-        <v>5.8754355922657897</v>
+        <v>5.8216366860907103</v>
       </c>
       <c r="D21" s="4">
         <v>1</v>
       </c>
       <c r="E21" s="5">
-        <v>26610.0854356729</v>
+        <v>25639.1304803313</v>
       </c>
       <c r="F21" s="5">
-        <v>26610.0854356729</v>
+        <v>25639.1304803313</v>
       </c>
       <c r="G21" s="5">
-        <v>156345.84308198601</v>
+        <v>149261.702603763</v>
       </c>
       <c r="H21" s="6">
         <v>0</v>
       </c>
       <c r="I21" s="5">
-        <v>156345.84308198601</v>
+        <v>149261.702603763</v>
       </c>
       <c r="J21" s="7">
-        <v>5.8754355922657897</v>
+        <v>5.8216366860907103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>